<commit_message>
Update financial_model_pivot_report.xlsx for w01_MBA_c1_out (1).xlsm
</commit_message>
<xml_diff>
--- a/financial_model_pivot_report.xlsx
+++ b/financial_model_pivot_report.xlsx
@@ -2375,12 +2375,6 @@
           <t>P61</t>
         </is>
       </c>
-      <c r="C122" t="n">
-        <v>386606</v>
-      </c>
-      <c r="D122" t="n">
-        <v>367910</v>
-      </c>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -2391,12 +2385,6 @@
           <t>P61</t>
         </is>
       </c>
-      <c r="C123" t="n">
-        <v>365571</v>
-      </c>
-      <c r="D123" t="n">
-        <v>366392</v>
-      </c>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -2407,12 +2395,6 @@
           <t>P62</t>
         </is>
       </c>
-      <c r="C124" t="n">
-        <v>381774</v>
-      </c>
-      <c r="D124" t="n">
-        <v>354291</v>
-      </c>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -2422,12 +2404,6 @@
         <is>
           <t>P62</t>
         </is>
-      </c>
-      <c r="C125" t="n">
-        <v>365570</v>
-      </c>
-      <c r="D125" t="n">
-        <v>389513</v>
       </c>
     </row>
     <row r="126">
@@ -25985,21 +25961,6 @@
           <t>P61</t>
         </is>
       </c>
-      <c r="D722" t="n">
-        <v>621618.8815449184</v>
-      </c>
-      <c r="E722" t="n">
-        <v>21312</v>
-      </c>
-      <c r="F722" t="n">
-        <v>1132200</v>
-      </c>
-      <c r="G722" t="n">
-        <v>416831.1184550816</v>
-      </c>
-      <c r="H722" t="n">
-        <v>93750</v>
-      </c>
     </row>
     <row r="723">
       <c r="A723" t="inlineStr">
@@ -26015,24 +25976,6 @@
           <t>P61</t>
         </is>
       </c>
-      <c r="D723" t="n">
-        <v>599564.3200646584</v>
-      </c>
-      <c r="E723" t="n">
-        <v>20475</v>
-      </c>
-      <c r="F723" t="n">
-        <v>1439648.4375</v>
-      </c>
-      <c r="G723" t="n">
-        <v>582636.4611853416</v>
-      </c>
-      <c r="H723" t="n">
-        <v>125000</v>
-      </c>
-      <c r="I723" t="n">
-        <v>132447.65625</v>
-      </c>
     </row>
     <row r="724">
       <c r="A724" t="inlineStr">
@@ -26048,24 +25991,6 @@
           <t>P61</t>
         </is>
       </c>
-      <c r="D724" t="n">
-        <v>1482322.533318183</v>
-      </c>
-      <c r="E724" t="n">
-        <v>54354</v>
-      </c>
-      <c r="F724" t="n">
-        <v>3275176.923076923</v>
-      </c>
-      <c r="G724" t="n">
-        <v>1095696.043604894</v>
-      </c>
-      <c r="H724" t="n">
-        <v>320513</v>
-      </c>
-      <c r="I724" t="n">
-        <v>376645.3461538462</v>
-      </c>
     </row>
     <row r="725">
       <c r="A725" t="inlineStr">
@@ -26081,24 +26006,6 @@
           <t>P61</t>
         </is>
       </c>
-      <c r="D725" t="n">
-        <v>1712218.776548889</v>
-      </c>
-      <c r="E725" t="n">
-        <v>63097</v>
-      </c>
-      <c r="F725" t="n">
-        <v>4449147.435897436</v>
-      </c>
-      <c r="G725" t="n">
-        <v>1776558.704220341</v>
-      </c>
-      <c r="H725" t="n">
-        <v>448718.0000000001</v>
-      </c>
-      <c r="I725" t="n">
-        <v>511651.9551282052</v>
-      </c>
     </row>
     <row r="726">
       <c r="A726" t="inlineStr">
@@ -26114,24 +26021,6 @@
           <t>P61</t>
         </is>
       </c>
-      <c r="D726" t="n">
-        <v>1349219.658410019</v>
-      </c>
-      <c r="E726" t="n">
-        <v>70595</v>
-      </c>
-      <c r="F726" t="n">
-        <v>3172808.988764046</v>
-      </c>
-      <c r="G726" t="n">
-        <v>1380733.521365263</v>
-      </c>
-      <c r="H726" t="n">
-        <v>157303</v>
-      </c>
-      <c r="I726" t="n">
-        <v>285552.8089887641</v>
-      </c>
     </row>
     <row r="727">
       <c r="A727" t="inlineStr">
@@ -26147,24 +26036,6 @@
           <t>P61</t>
         </is>
       </c>
-      <c r="D727" t="n">
-        <v>1924729.465013138</v>
-      </c>
-      <c r="E727" t="n">
-        <v>62384</v>
-      </c>
-      <c r="F727" t="n">
-        <v>4275757.303370787</v>
-      </c>
-      <c r="G727" t="n">
-        <v>1775198.681054278</v>
-      </c>
-      <c r="H727" t="n">
-        <v>191011</v>
-      </c>
-      <c r="I727" t="n">
-        <v>384818.1573033708</v>
-      </c>
     </row>
     <row r="728">
       <c r="A728" t="inlineStr">
@@ -26180,24 +26051,6 @@
           <t>P61</t>
         </is>
       </c>
-      <c r="D728" t="n">
-        <v>129573.8958258609</v>
-      </c>
-      <c r="E728" t="n">
-        <v>32520</v>
-      </c>
-      <c r="F728" t="n">
-        <v>914625</v>
-      </c>
-      <c r="G728" t="n">
-        <v>675066.9791741391</v>
-      </c>
-      <c r="H728" t="n">
-        <v>46875</v>
-      </c>
-      <c r="I728" t="n">
-        <v>63109.12499999999</v>
-      </c>
     </row>
     <row r="729">
       <c r="A729" t="inlineStr">
@@ -26213,21 +26066,6 @@
           <t>P61</t>
         </is>
       </c>
-      <c r="D729" t="n">
-        <v>116553.3980360625</v>
-      </c>
-      <c r="E729" t="n">
-        <v>24527</v>
-      </c>
-      <c r="F729" t="n">
-        <v>862277.34375</v>
-      </c>
-      <c r="G729" t="n">
-        <v>683223.9457139375</v>
-      </c>
-      <c r="H729" t="n">
-        <v>62500</v>
-      </c>
     </row>
     <row r="730">
       <c r="A730" t="inlineStr">
@@ -26243,24 +26081,6 @@
           <t>P61</t>
         </is>
       </c>
-      <c r="D730" t="n">
-        <v>760049.5659322058</v>
-      </c>
-      <c r="E730" t="n">
-        <v>49197</v>
-      </c>
-      <c r="F730" t="n">
-        <v>2236227.272727272</v>
-      </c>
-      <c r="G730" t="n">
-        <v>991738.5704314305</v>
-      </c>
-      <c r="H730" t="n">
-        <v>227273</v>
-      </c>
-      <c r="I730" t="n">
-        <v>257166.1363636364</v>
-      </c>
     </row>
     <row r="731">
       <c r="A731" t="inlineStr">
@@ -26276,24 +26096,6 @@
           <t>P61</t>
         </is>
       </c>
-      <c r="D731" t="n">
-        <v>964541.9870886491</v>
-      </c>
-      <c r="E731" t="n">
-        <v>49747</v>
-      </c>
-      <c r="F731" t="n">
-        <v>3014969.696969697</v>
-      </c>
-      <c r="G731" t="n">
-        <v>1400676.194729533</v>
-      </c>
-      <c r="H731" t="n">
-        <v>303030</v>
-      </c>
-      <c r="I731" t="n">
-        <v>346721.5151515151</v>
-      </c>
     </row>
     <row r="732">
       <c r="A732" t="inlineStr">
@@ -26309,24 +26111,6 @@
           <t>P61</t>
         </is>
       </c>
-      <c r="D732" t="n">
-        <v>1850272.501900503</v>
-      </c>
-      <c r="E732" t="n">
-        <v>139932</v>
-      </c>
-      <c r="F732" t="n">
-        <v>6017076</v>
-      </c>
-      <c r="G732" t="n">
-        <v>2820821.628099496</v>
-      </c>
-      <c r="H732" t="n">
-        <v>1000000</v>
-      </c>
-      <c r="I732" t="n">
-        <v>345981.87</v>
-      </c>
     </row>
     <row r="733">
       <c r="A733" t="inlineStr">
@@ -26342,21 +26126,6 @@
           <t>P61</t>
         </is>
       </c>
-      <c r="D733" t="n">
-        <v>2913584.31893666</v>
-      </c>
-      <c r="E733" t="n">
-        <v>146162</v>
-      </c>
-      <c r="F733" t="n">
-        <v>8185072</v>
-      </c>
-      <c r="G733" t="n">
-        <v>4071487.68106334</v>
-      </c>
-      <c r="H733" t="n">
-        <v>1200000</v>
-      </c>
     </row>
     <row r="734">
       <c r="A734" t="inlineStr">
@@ -26372,21 +26141,6 @@
           <t>P62</t>
         </is>
       </c>
-      <c r="D734" t="n">
-        <v>612818.8971076387</v>
-      </c>
-      <c r="E734" t="n">
-        <v>21253</v>
-      </c>
-      <c r="F734" t="n">
-        <v>1111695.384615385</v>
-      </c>
-      <c r="G734" t="n">
-        <v>406568.4875077458</v>
-      </c>
-      <c r="H734" t="n">
-        <v>92308</v>
-      </c>
     </row>
     <row r="735">
       <c r="A735" t="inlineStr">
@@ -26402,24 +26156,6 @@
           <t>P62</t>
         </is>
       </c>
-      <c r="D735" t="n">
-        <v>668285.0635329934</v>
-      </c>
-      <c r="E735" t="n">
-        <v>22786</v>
-      </c>
-      <c r="F735" t="n">
-        <v>1577492.307692308</v>
-      </c>
-      <c r="G735" t="n">
-        <v>628692.9518516217</v>
-      </c>
-      <c r="H735" t="n">
-        <v>135385</v>
-      </c>
-      <c r="I735" t="n">
-        <v>145129.2923076923</v>
-      </c>
     </row>
     <row r="736">
       <c r="A736" t="inlineStr">
@@ -26435,24 +26171,6 @@
           <t>P62</t>
         </is>
       </c>
-      <c r="D736" t="n">
-        <v>1452689.353788959</v>
-      </c>
-      <c r="E736" t="n">
-        <v>51834</v>
-      </c>
-      <c r="F736" t="n">
-        <v>3163893.506493506</v>
-      </c>
-      <c r="G736" t="n">
-        <v>1022681.399457794</v>
-      </c>
-      <c r="H736" t="n">
-        <v>324675</v>
-      </c>
-      <c r="I736" t="n">
-        <v>363847.7532467532</v>
-      </c>
     </row>
     <row r="737">
       <c r="A737" t="inlineStr">
@@ -26468,24 +26186,6 @@
           <t>P62</t>
         </is>
       </c>
-      <c r="D737" t="n">
-        <v>1815893.782519003</v>
-      </c>
-      <c r="E737" t="n">
-        <v>65387</v>
-      </c>
-      <c r="F737" t="n">
-        <v>4670500</v>
-      </c>
-      <c r="G737" t="n">
-        <v>1862953.717480996</v>
-      </c>
-      <c r="H737" t="n">
-        <v>454545</v>
-      </c>
-      <c r="I737" t="n">
-        <v>537107.5</v>
-      </c>
     </row>
     <row r="738">
       <c r="A738" t="inlineStr">
@@ -26501,24 +26201,6 @@
           <t>P62</t>
         </is>
       </c>
-      <c r="D738" t="n">
-        <v>1417305.668512515</v>
-      </c>
-      <c r="E738" t="n">
-        <v>73793</v>
-      </c>
-      <c r="F738" t="n">
-        <v>3279688.888888889</v>
-      </c>
-      <c r="G738" t="n">
-        <v>1411655.220376374</v>
-      </c>
-      <c r="H738" t="n">
-        <v>155556</v>
-      </c>
-      <c r="I738" t="n">
-        <v>295172</v>
-      </c>
     </row>
     <row r="739">
       <c r="A739" t="inlineStr">
@@ -26534,21 +26216,6 @@
           <t>P62</t>
         </is>
       </c>
-      <c r="D739" t="n">
-        <v>2465193.723461791</v>
-      </c>
-      <c r="E739" t="n">
-        <v>66044</v>
-      </c>
-      <c r="F739" t="n">
-        <v>4476315.555555555</v>
-      </c>
-      <c r="G739" t="n">
-        <v>1822232.832093764</v>
-      </c>
-      <c r="H739" t="n">
-        <v>188889</v>
-      </c>
     </row>
     <row r="740">
       <c r="A740" t="inlineStr">
@@ -26564,24 +26231,6 @@
           <t>P62</t>
         </is>
       </c>
-      <c r="D740" t="n">
-        <v>133494.4724707446</v>
-      </c>
-      <c r="E740" t="n">
-        <v>30809</v>
-      </c>
-      <c r="F740" t="n">
-        <v>866503.125</v>
-      </c>
-      <c r="G740" t="n">
-        <v>626344.9369042554</v>
-      </c>
-      <c r="H740" t="n">
-        <v>46875</v>
-      </c>
-      <c r="I740" t="n">
-        <v>59788.71562499999</v>
-      </c>
     </row>
     <row r="741">
       <c r="A741" t="inlineStr">
@@ -26597,24 +26246,6 @@
           <t>P62</t>
         </is>
       </c>
-      <c r="D741" t="n">
-        <v>38530.63286774315</v>
-      </c>
-      <c r="E741" t="n">
-        <v>22257</v>
-      </c>
-      <c r="F741" t="n">
-        <v>782472.65625</v>
-      </c>
-      <c r="G741" t="n">
-        <v>627451.4101010069</v>
-      </c>
-      <c r="H741" t="n">
-        <v>62500</v>
-      </c>
-      <c r="I741" t="n">
-        <v>53990.61328124999</v>
-      </c>
     </row>
     <row r="742">
       <c r="A742" t="inlineStr">
@@ -26630,24 +26261,6 @@
           <t>P62</t>
         </is>
       </c>
-      <c r="D742" t="n">
-        <v>796197.2355270309</v>
-      </c>
-      <c r="E742" t="n">
-        <v>48634</v>
-      </c>
-      <c r="F742" t="n">
-        <v>2244646.153846154</v>
-      </c>
-      <c r="G742" t="n">
-        <v>959545.6106268154</v>
-      </c>
-      <c r="H742" t="n">
-        <v>230769</v>
-      </c>
-      <c r="I742" t="n">
-        <v>258134.3076923077</v>
-      </c>
     </row>
     <row r="743">
       <c r="A743" t="inlineStr">
@@ -26663,24 +26276,6 @@
           <t>P62</t>
         </is>
       </c>
-      <c r="D743" t="n">
-        <v>1124187.786806732</v>
-      </c>
-      <c r="E743" t="n">
-        <v>56320</v>
-      </c>
-      <c r="F743" t="n">
-        <v>3465846.153846154</v>
-      </c>
-      <c r="G743" t="n">
-        <v>1604624.059347114</v>
-      </c>
-      <c r="H743" t="n">
-        <v>338462</v>
-      </c>
-      <c r="I743" t="n">
-        <v>398572.3076923077</v>
-      </c>
     </row>
     <row r="744">
       <c r="A744" t="inlineStr">
@@ -26696,24 +26291,6 @@
           <t>P62</t>
         </is>
       </c>
-      <c r="D744" t="n">
-        <v>1661422.924649169</v>
-      </c>
-      <c r="E744" t="n">
-        <v>127968</v>
-      </c>
-      <c r="F744" t="n">
-        <v>5502624</v>
-      </c>
-      <c r="G744" t="n">
-        <v>2524800.195350831</v>
-      </c>
-      <c r="H744" t="n">
-        <v>1000000</v>
-      </c>
-      <c r="I744" t="n">
-        <v>316400.88</v>
-      </c>
     </row>
     <row r="745">
       <c r="A745" t="inlineStr">
@@ -26728,24 +26305,6 @@
         <is>
           <t>P62</t>
         </is>
-      </c>
-      <c r="D745" t="n">
-        <v>2653533.05059623</v>
-      </c>
-      <c r="E745" t="n">
-        <v>156719</v>
-      </c>
-      <c r="F745" t="n">
-        <v>8776264</v>
-      </c>
-      <c r="G745" t="n">
-        <v>4418095.76940377</v>
-      </c>
-      <c r="H745" t="n">
-        <v>1200000</v>
-      </c>
-      <c r="I745" t="n">
-        <v>504635.18</v>
       </c>
     </row>
     <row r="746">

</xml_diff>

<commit_message>
Update financial_model_pivot_report.xlsx for w01_MBA_c1_out (2).xlsm
</commit_message>
<xml_diff>
--- a/financial_model_pivot_report.xlsx
+++ b/financial_model_pivot_report.xlsx
@@ -2375,6 +2375,12 @@
           <t>P61</t>
         </is>
       </c>
+      <c r="C122" t="n">
+        <v>386606</v>
+      </c>
+      <c r="D122" t="n">
+        <v>367910</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -2385,6 +2391,12 @@
           <t>P61</t>
         </is>
       </c>
+      <c r="C123" t="n">
+        <v>365571</v>
+      </c>
+      <c r="D123" t="n">
+        <v>366392</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -2395,6 +2407,12 @@
           <t>P62</t>
         </is>
       </c>
+      <c r="C124" t="n">
+        <v>381774</v>
+      </c>
+      <c r="D124" t="n">
+        <v>354291</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -2404,6 +2422,12 @@
         <is>
           <t>P62</t>
         </is>
+      </c>
+      <c r="C125" t="n">
+        <v>365570</v>
+      </c>
+      <c r="D125" t="n">
+        <v>389513</v>
       </c>
     </row>
     <row r="126">
@@ -25961,6 +25985,21 @@
           <t>P61</t>
         </is>
       </c>
+      <c r="D722" t="n">
+        <v>621618.8815449184</v>
+      </c>
+      <c r="E722" t="n">
+        <v>21312</v>
+      </c>
+      <c r="F722" t="n">
+        <v>1132200</v>
+      </c>
+      <c r="G722" t="n">
+        <v>416831.1184550816</v>
+      </c>
+      <c r="H722" t="n">
+        <v>93750</v>
+      </c>
     </row>
     <row r="723">
       <c r="A723" t="inlineStr">
@@ -25976,6 +26015,24 @@
           <t>P61</t>
         </is>
       </c>
+      <c r="D723" t="n">
+        <v>599564.3200646584</v>
+      </c>
+      <c r="E723" t="n">
+        <v>20475</v>
+      </c>
+      <c r="F723" t="n">
+        <v>1439648.4375</v>
+      </c>
+      <c r="G723" t="n">
+        <v>582636.4611853416</v>
+      </c>
+      <c r="H723" t="n">
+        <v>125000</v>
+      </c>
+      <c r="I723" t="n">
+        <v>132447.65625</v>
+      </c>
     </row>
     <row r="724">
       <c r="A724" t="inlineStr">
@@ -25991,6 +26048,24 @@
           <t>P61</t>
         </is>
       </c>
+      <c r="D724" t="n">
+        <v>1482322.533318183</v>
+      </c>
+      <c r="E724" t="n">
+        <v>54354</v>
+      </c>
+      <c r="F724" t="n">
+        <v>3275176.923076923</v>
+      </c>
+      <c r="G724" t="n">
+        <v>1095696.043604894</v>
+      </c>
+      <c r="H724" t="n">
+        <v>320513</v>
+      </c>
+      <c r="I724" t="n">
+        <v>376645.3461538462</v>
+      </c>
     </row>
     <row r="725">
       <c r="A725" t="inlineStr">
@@ -26006,6 +26081,24 @@
           <t>P61</t>
         </is>
       </c>
+      <c r="D725" t="n">
+        <v>1712218.776548889</v>
+      </c>
+      <c r="E725" t="n">
+        <v>63097</v>
+      </c>
+      <c r="F725" t="n">
+        <v>4449147.435897436</v>
+      </c>
+      <c r="G725" t="n">
+        <v>1776558.704220341</v>
+      </c>
+      <c r="H725" t="n">
+        <v>448718.0000000001</v>
+      </c>
+      <c r="I725" t="n">
+        <v>511651.9551282052</v>
+      </c>
     </row>
     <row r="726">
       <c r="A726" t="inlineStr">
@@ -26021,6 +26114,24 @@
           <t>P61</t>
         </is>
       </c>
+      <c r="D726" t="n">
+        <v>1349219.658410019</v>
+      </c>
+      <c r="E726" t="n">
+        <v>70595</v>
+      </c>
+      <c r="F726" t="n">
+        <v>3172808.988764046</v>
+      </c>
+      <c r="G726" t="n">
+        <v>1380733.521365263</v>
+      </c>
+      <c r="H726" t="n">
+        <v>157303</v>
+      </c>
+      <c r="I726" t="n">
+        <v>285552.8089887641</v>
+      </c>
     </row>
     <row r="727">
       <c r="A727" t="inlineStr">
@@ -26036,6 +26147,24 @@
           <t>P61</t>
         </is>
       </c>
+      <c r="D727" t="n">
+        <v>1924729.465013138</v>
+      </c>
+      <c r="E727" t="n">
+        <v>62384</v>
+      </c>
+      <c r="F727" t="n">
+        <v>4275757.303370787</v>
+      </c>
+      <c r="G727" t="n">
+        <v>1775198.681054278</v>
+      </c>
+      <c r="H727" t="n">
+        <v>191011</v>
+      </c>
+      <c r="I727" t="n">
+        <v>384818.1573033708</v>
+      </c>
     </row>
     <row r="728">
       <c r="A728" t="inlineStr">
@@ -26051,6 +26180,24 @@
           <t>P61</t>
         </is>
       </c>
+      <c r="D728" t="n">
+        <v>129573.8958258609</v>
+      </c>
+      <c r="E728" t="n">
+        <v>32520</v>
+      </c>
+      <c r="F728" t="n">
+        <v>914625</v>
+      </c>
+      <c r="G728" t="n">
+        <v>675066.9791741391</v>
+      </c>
+      <c r="H728" t="n">
+        <v>46875</v>
+      </c>
+      <c r="I728" t="n">
+        <v>63109.12499999999</v>
+      </c>
     </row>
     <row r="729">
       <c r="A729" t="inlineStr">
@@ -26066,6 +26213,21 @@
           <t>P61</t>
         </is>
       </c>
+      <c r="D729" t="n">
+        <v>116553.3980360625</v>
+      </c>
+      <c r="E729" t="n">
+        <v>24527</v>
+      </c>
+      <c r="F729" t="n">
+        <v>862277.34375</v>
+      </c>
+      <c r="G729" t="n">
+        <v>683223.9457139375</v>
+      </c>
+      <c r="H729" t="n">
+        <v>62500</v>
+      </c>
     </row>
     <row r="730">
       <c r="A730" t="inlineStr">
@@ -26081,6 +26243,24 @@
           <t>P61</t>
         </is>
       </c>
+      <c r="D730" t="n">
+        <v>760049.5659322058</v>
+      </c>
+      <c r="E730" t="n">
+        <v>49197</v>
+      </c>
+      <c r="F730" t="n">
+        <v>2236227.272727272</v>
+      </c>
+      <c r="G730" t="n">
+        <v>991738.5704314305</v>
+      </c>
+      <c r="H730" t="n">
+        <v>227273</v>
+      </c>
+      <c r="I730" t="n">
+        <v>257166.1363636364</v>
+      </c>
     </row>
     <row r="731">
       <c r="A731" t="inlineStr">
@@ -26096,6 +26276,24 @@
           <t>P61</t>
         </is>
       </c>
+      <c r="D731" t="n">
+        <v>964541.9870886491</v>
+      </c>
+      <c r="E731" t="n">
+        <v>49747</v>
+      </c>
+      <c r="F731" t="n">
+        <v>3014969.696969697</v>
+      </c>
+      <c r="G731" t="n">
+        <v>1400676.194729533</v>
+      </c>
+      <c r="H731" t="n">
+        <v>303030</v>
+      </c>
+      <c r="I731" t="n">
+        <v>346721.5151515151</v>
+      </c>
     </row>
     <row r="732">
       <c r="A732" t="inlineStr">
@@ -26111,6 +26309,24 @@
           <t>P61</t>
         </is>
       </c>
+      <c r="D732" t="n">
+        <v>1850272.501900503</v>
+      </c>
+      <c r="E732" t="n">
+        <v>139932</v>
+      </c>
+      <c r="F732" t="n">
+        <v>6017076</v>
+      </c>
+      <c r="G732" t="n">
+        <v>2820821.628099496</v>
+      </c>
+      <c r="H732" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="I732" t="n">
+        <v>345981.87</v>
+      </c>
     </row>
     <row r="733">
       <c r="A733" t="inlineStr">
@@ -26126,6 +26342,21 @@
           <t>P61</t>
         </is>
       </c>
+      <c r="D733" t="n">
+        <v>2913584.31893666</v>
+      </c>
+      <c r="E733" t="n">
+        <v>146162</v>
+      </c>
+      <c r="F733" t="n">
+        <v>8185072</v>
+      </c>
+      <c r="G733" t="n">
+        <v>4071487.68106334</v>
+      </c>
+      <c r="H733" t="n">
+        <v>1200000</v>
+      </c>
     </row>
     <row r="734">
       <c r="A734" t="inlineStr">
@@ -26141,6 +26372,21 @@
           <t>P62</t>
         </is>
       </c>
+      <c r="D734" t="n">
+        <v>612818.8971076387</v>
+      </c>
+      <c r="E734" t="n">
+        <v>21253</v>
+      </c>
+      <c r="F734" t="n">
+        <v>1111695.384615385</v>
+      </c>
+      <c r="G734" t="n">
+        <v>406568.4875077458</v>
+      </c>
+      <c r="H734" t="n">
+        <v>92308</v>
+      </c>
     </row>
     <row r="735">
       <c r="A735" t="inlineStr">
@@ -26156,6 +26402,24 @@
           <t>P62</t>
         </is>
       </c>
+      <c r="D735" t="n">
+        <v>668285.0635329934</v>
+      </c>
+      <c r="E735" t="n">
+        <v>22786</v>
+      </c>
+      <c r="F735" t="n">
+        <v>1577492.307692308</v>
+      </c>
+      <c r="G735" t="n">
+        <v>628692.9518516217</v>
+      </c>
+      <c r="H735" t="n">
+        <v>135385</v>
+      </c>
+      <c r="I735" t="n">
+        <v>145129.2923076923</v>
+      </c>
     </row>
     <row r="736">
       <c r="A736" t="inlineStr">
@@ -26171,6 +26435,24 @@
           <t>P62</t>
         </is>
       </c>
+      <c r="D736" t="n">
+        <v>1452689.353788959</v>
+      </c>
+      <c r="E736" t="n">
+        <v>51834</v>
+      </c>
+      <c r="F736" t="n">
+        <v>3163893.506493506</v>
+      </c>
+      <c r="G736" t="n">
+        <v>1022681.399457794</v>
+      </c>
+      <c r="H736" t="n">
+        <v>324675</v>
+      </c>
+      <c r="I736" t="n">
+        <v>363847.7532467532</v>
+      </c>
     </row>
     <row r="737">
       <c r="A737" t="inlineStr">
@@ -26186,6 +26468,24 @@
           <t>P62</t>
         </is>
       </c>
+      <c r="D737" t="n">
+        <v>1815893.782519003</v>
+      </c>
+      <c r="E737" t="n">
+        <v>65387</v>
+      </c>
+      <c r="F737" t="n">
+        <v>4670500</v>
+      </c>
+      <c r="G737" t="n">
+        <v>1862953.717480996</v>
+      </c>
+      <c r="H737" t="n">
+        <v>454545</v>
+      </c>
+      <c r="I737" t="n">
+        <v>537107.5</v>
+      </c>
     </row>
     <row r="738">
       <c r="A738" t="inlineStr">
@@ -26201,6 +26501,24 @@
           <t>P62</t>
         </is>
       </c>
+      <c r="D738" t="n">
+        <v>1417305.668512515</v>
+      </c>
+      <c r="E738" t="n">
+        <v>73793</v>
+      </c>
+      <c r="F738" t="n">
+        <v>3279688.888888889</v>
+      </c>
+      <c r="G738" t="n">
+        <v>1411655.220376374</v>
+      </c>
+      <c r="H738" t="n">
+        <v>155556</v>
+      </c>
+      <c r="I738" t="n">
+        <v>295172</v>
+      </c>
     </row>
     <row r="739">
       <c r="A739" t="inlineStr">
@@ -26216,6 +26534,21 @@
           <t>P62</t>
         </is>
       </c>
+      <c r="D739" t="n">
+        <v>2465193.723461791</v>
+      </c>
+      <c r="E739" t="n">
+        <v>66044</v>
+      </c>
+      <c r="F739" t="n">
+        <v>4476315.555555555</v>
+      </c>
+      <c r="G739" t="n">
+        <v>1822232.832093764</v>
+      </c>
+      <c r="H739" t="n">
+        <v>188889</v>
+      </c>
     </row>
     <row r="740">
       <c r="A740" t="inlineStr">
@@ -26231,6 +26564,24 @@
           <t>P62</t>
         </is>
       </c>
+      <c r="D740" t="n">
+        <v>133494.4724707446</v>
+      </c>
+      <c r="E740" t="n">
+        <v>30809</v>
+      </c>
+      <c r="F740" t="n">
+        <v>866503.125</v>
+      </c>
+      <c r="G740" t="n">
+        <v>626344.9369042554</v>
+      </c>
+      <c r="H740" t="n">
+        <v>46875</v>
+      </c>
+      <c r="I740" t="n">
+        <v>59788.71562499999</v>
+      </c>
     </row>
     <row r="741">
       <c r="A741" t="inlineStr">
@@ -26246,6 +26597,24 @@
           <t>P62</t>
         </is>
       </c>
+      <c r="D741" t="n">
+        <v>38530.63286774315</v>
+      </c>
+      <c r="E741" t="n">
+        <v>22257</v>
+      </c>
+      <c r="F741" t="n">
+        <v>782472.65625</v>
+      </c>
+      <c r="G741" t="n">
+        <v>627451.4101010069</v>
+      </c>
+      <c r="H741" t="n">
+        <v>62500</v>
+      </c>
+      <c r="I741" t="n">
+        <v>53990.61328124999</v>
+      </c>
     </row>
     <row r="742">
       <c r="A742" t="inlineStr">
@@ -26261,6 +26630,24 @@
           <t>P62</t>
         </is>
       </c>
+      <c r="D742" t="n">
+        <v>796197.2355270309</v>
+      </c>
+      <c r="E742" t="n">
+        <v>48634</v>
+      </c>
+      <c r="F742" t="n">
+        <v>2244646.153846154</v>
+      </c>
+      <c r="G742" t="n">
+        <v>959545.6106268154</v>
+      </c>
+      <c r="H742" t="n">
+        <v>230769</v>
+      </c>
+      <c r="I742" t="n">
+        <v>258134.3076923077</v>
+      </c>
     </row>
     <row r="743">
       <c r="A743" t="inlineStr">
@@ -26276,6 +26663,24 @@
           <t>P62</t>
         </is>
       </c>
+      <c r="D743" t="n">
+        <v>1124187.786806732</v>
+      </c>
+      <c r="E743" t="n">
+        <v>56320</v>
+      </c>
+      <c r="F743" t="n">
+        <v>3465846.153846154</v>
+      </c>
+      <c r="G743" t="n">
+        <v>1604624.059347114</v>
+      </c>
+      <c r="H743" t="n">
+        <v>338462</v>
+      </c>
+      <c r="I743" t="n">
+        <v>398572.3076923077</v>
+      </c>
     </row>
     <row r="744">
       <c r="A744" t="inlineStr">
@@ -26291,6 +26696,24 @@
           <t>P62</t>
         </is>
       </c>
+      <c r="D744" t="n">
+        <v>1661422.924649169</v>
+      </c>
+      <c r="E744" t="n">
+        <v>127968</v>
+      </c>
+      <c r="F744" t="n">
+        <v>5502624</v>
+      </c>
+      <c r="G744" t="n">
+        <v>2524800.195350831</v>
+      </c>
+      <c r="H744" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="I744" t="n">
+        <v>316400.88</v>
+      </c>
     </row>
     <row r="745">
       <c r="A745" t="inlineStr">
@@ -26305,6 +26728,24 @@
         <is>
           <t>P62</t>
         </is>
+      </c>
+      <c r="D745" t="n">
+        <v>2653533.05059623</v>
+      </c>
+      <c r="E745" t="n">
+        <v>156719</v>
+      </c>
+      <c r="F745" t="n">
+        <v>8776264</v>
+      </c>
+      <c r="G745" t="n">
+        <v>4418095.76940377</v>
+      </c>
+      <c r="H745" t="n">
+        <v>1200000</v>
+      </c>
+      <c r="I745" t="n">
+        <v>504635.18</v>
       </c>
     </row>
     <row r="746">

</xml_diff>